<commit_message>
fixing the error and spacings in CustomException file activity and adding to the exce file compilations
</commit_message>
<xml_diff>
--- a/activities_compilation.xlsx
+++ b/activities_compilation.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OOPROG21\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBD8B728-C9DA-4D7E-8499-EEAE7255F67C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7755"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="19">
   <si>
     <t>Date</t>
   </si>
@@ -62,16 +63,31 @@
     <t>University Payment System</t>
   </si>
   <si>
-    <t>Oct. 19, 2026</t>
-  </si>
-  <si>
     <t>Sept. 30</t>
+  </si>
+  <si>
+    <t>Sept. 28</t>
+  </si>
+  <si>
+    <t>Oct. 2</t>
+  </si>
+  <si>
+    <t>Oct. 16</t>
+  </si>
+  <si>
+    <t>Oct. 21</t>
+  </si>
+  <si>
+    <t>Custom Exception</t>
+  </si>
+  <si>
+    <t>Oct. 19</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -89,7 +105,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -175,19 +191,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -252,7 +255,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -263,52 +266,49 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -590,191 +590,215 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="36.140625" style="1" customWidth="1"/>
-    <col min="3" max="4" width="9.140625" style="1"/>
-    <col min="5" max="5" width="18.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7265625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="36.1796875" style="1" customWidth="1"/>
+    <col min="3" max="4" width="9.1796875" style="1"/>
+    <col min="5" max="5" width="18.453125" style="1" customWidth="1"/>
     <col min="6" max="6" width="18" style="1" customWidth="1"/>
     <col min="7" max="7" width="13" style="1" customWidth="1"/>
-    <col min="8" max="9" width="9.140625" style="1"/>
+    <col min="8" max="9" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="19"/>
+      <c r="D1" s="11"/>
       <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="3" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="4"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="I1" s="12"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="14" t="s">
+      <c r="C2" s="13"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="2"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="14"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="9"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="2"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="15"/>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="15" t="s">
+      <c r="C3" s="15"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="4"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="16"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="10"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="11"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="15"/>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="15"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="4"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="16"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="15"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="4"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="16"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="11"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="11"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="15"/>
-      <c r="B6" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="11"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="15"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="11"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="15"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="11"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="15"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="11"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="15"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="11"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="15"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="11"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="12"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="4"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="16"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="15"/>
+      <c r="D7" s="16"/>
+      <c r="E7" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="7"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="16"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="7"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="16"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="7"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="16"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="16"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="7"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="16"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" s="8"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H9:I9"/>
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="H11:I11"/>
     <mergeCell ref="H12:I12"/>
@@ -788,15 +812,17 @@
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="H7:I7"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H9:I9"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="H1:I1"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
putting the gui student resgistration to excel tracking
</commit_message>
<xml_diff>
--- a/activities_compilation.xlsx
+++ b/activities_compilation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OOPROG21\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBD8B728-C9DA-4D7E-8499-EEAE7255F67C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEAF96F7-5A7B-4C69-BE03-840134C29E77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="1520" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="21">
   <si>
     <t>Date</t>
   </si>
@@ -82,6 +82,12 @@
   </si>
   <si>
     <t>Oct. 19</t>
+  </si>
+  <si>
+    <t>Oct. 23</t>
+  </si>
+  <si>
+    <t>GUI Student Registration</t>
   </si>
 </sst>
 </file>
@@ -284,6 +290,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -291,24 +315,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -592,28 +598,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.7265625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="36.1796875" style="1" customWidth="1"/>
-    <col min="3" max="4" width="9.1796875" style="1"/>
-    <col min="5" max="5" width="18.453125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="16.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="36.140625" style="1" customWidth="1"/>
+    <col min="3" max="4" width="9.140625" style="1"/>
+    <col min="5" max="5" width="18.42578125" style="1" customWidth="1"/>
     <col min="6" max="6" width="18" style="1" customWidth="1"/>
     <col min="7" max="7" width="13" style="1" customWidth="1"/>
-    <col min="8" max="9" width="9.1796875" style="1"/>
+    <col min="8" max="9" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="11"/>
+      <c r="D1" s="17"/>
       <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
@@ -623,20 +629,20 @@
       <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="12"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="I1" s="18"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>13</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="13"/>
-      <c r="D2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="15"/>
       <c r="E2" s="6" t="s">
         <v>18</v>
       </c>
@@ -644,18 +650,18 @@
         <v>16</v>
       </c>
       <c r="G2" s="2"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="14"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H2" s="14"/>
+      <c r="I2" s="15"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="16"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="11"/>
       <c r="E3" s="7" t="s">
         <v>18</v>
       </c>
@@ -663,18 +669,18 @@
         <v>16</v>
       </c>
       <c r="G3" s="4"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="16"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H3" s="10"/>
+      <c r="I3" s="11"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="15"/>
-      <c r="D4" s="16"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="11"/>
       <c r="E4" s="7" t="s">
         <v>18</v>
       </c>
@@ -682,18 +688,18 @@
         <v>16</v>
       </c>
       <c r="G4" s="4"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="16"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H4" s="10"/>
+      <c r="I4" s="11"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>14</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="16"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="11"/>
       <c r="E5" s="7" t="s">
         <v>18</v>
       </c>
@@ -701,18 +707,18 @@
         <v>16</v>
       </c>
       <c r="G5" s="4"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="16"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H5" s="10"/>
+      <c r="I5" s="11"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>15</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="16"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="11"/>
       <c r="E6" s="7" t="s">
         <v>18</v>
       </c>
@@ -720,18 +726,18 @@
         <v>16</v>
       </c>
       <c r="G6" s="4"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="16"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H6" s="10"/>
+      <c r="I6" s="11"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>16</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="15"/>
-      <c r="D7" s="16"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="11"/>
       <c r="E7" s="7" t="s">
         <v>16</v>
       </c>
@@ -739,66 +745,90 @@
         <v>16</v>
       </c>
       <c r="G7" s="7"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="16"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="11"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="10"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>19</v>
+      </c>
       <c r="G8" s="7"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="16"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H8" s="10"/>
+      <c r="I8" s="11"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="16"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="11"/>
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="16"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H9" s="10"/>
+      <c r="I9" s="11"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="7"/>
       <c r="B10" s="7"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="16"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="11"/>
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
       <c r="G10" s="7"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="16"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H10" s="10"/>
+      <c r="I10" s="11"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="7"/>
       <c r="B11" s="7"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="16"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="11"/>
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
       <c r="G11" s="7"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="16"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="H11" s="10"/>
+      <c r="I11" s="11"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="18"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="13"/>
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="18"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="H11:I11"/>
     <mergeCell ref="H12:I12"/>
@@ -806,23 +836,7 @@
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="H8:I8"/>
     <mergeCell ref="H9:I9"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>